<commit_message>
added llm provider functionality for switching from openai to gemini
</commit_message>
<xml_diff>
--- a/input/test_flow.xlsx
+++ b/input/test_flow.xlsx
@@ -457,40 +457,40 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TC-UM-001</v>
+        <v>TC-UM-003</v>
       </c>
       <c r="B2" t="str">
-        <v>Verify successful manual user creation</v>
+        <v>Verify role assignment to user</v>
       </c>
       <c r="C2" t="str">
         <v>User Management</v>
       </c>
       <c r="D2" t="str">
-        <v>User Creation &amp; Invitations</v>
+        <v>Role Assignment</v>
       </c>
       <c r="E2" t="str">
-        <v>FSD ID FS-RL-CF-04: Client admin can create users within license limits</v>
+        <v>FSD ID FS-RL-CF-04: Roles must be assigned to users appropriately.</v>
       </c>
       <c r="F2" t="str">
-        <v>To ensure that a Client admin can create a new user manually.</v>
+        <v>To ensure a Client admin can assign a role to a user.</v>
       </c>
       <c r="G2" t="str">
-        <v>1. Client admin is logged in.; 2. Permissions for user creation are granted.</v>
+        <v>1. User is created and exists in the system.; 2. Administrator is logged in and viewing user details.</v>
       </c>
       <c r="H2" t="str">
-        <v>['Full Name: Text (max 50 chars, alphabets and spaces only)', 'Email Address: Text (max 100 chars, must be unique and valid format)', 'Role: Dropdown (must exist in Role Management)']</v>
+        <v>['Role: Dropdown (must exist in Role Management)']</v>
       </c>
       <c r="I2" t="str">
-        <v>1. Navigate to User Management; 2. Click on Add User and click New Internal User; 3. Enter first Name and last Name; 4. Enter Email Address; 5. Select Role; 6. Click on Save</v>
+        <v>1. Navigate to User Management; 2.Click on the user and click on menu and select edit.; 3. Select role from Role dropdown; 4. Click on Save.</v>
       </c>
       <c r="J2" t="str">
-        <v>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Full Name field shows the entered value.; 4. Email Address field shows the entered value.; 5. Role dropdown reflects the chosen role.; 6. User is visible in the list with correct status with status Pending.; Overall: New user is listed in User Management with Pending status.</v>
+        <v>1. User Management page is displayed.; 2. User details are displayed.; 3. Role dropdown reflects the chosen role.; 4. User role is updated successfully.; Overall: User's assigned role reflects changes in the user list.</v>
       </c>
       <c r="K2" t="str">
-        <v>User appears in the user list with status Pending.</v>
+        <v>User role matches the assigned role.</v>
       </c>
       <c r="L2" t="str">
-        <v>User is not listed or has an incorrect status.</v>
+        <v>User role is not updated in the user details.</v>
       </c>
       <c r="M2" t="str">
         <v>Functional - Positive</v>
@@ -502,7 +502,7 @@
         <v>Functional suitability</v>
       </c>
       <c r="P2" t="str">
-        <v>High</v>
+        <v>Medium</v>
       </c>
       <c r="Q2" t="str">
         <v>Yes</v>

</xml_diff>

<commit_message>
feat: introduce dynamic scenario runner and add configurable XPath locator policy
</commit_message>
<xml_diff>
--- a/input/test_flow.xlsx
+++ b/input/test_flow.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:R2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -457,10 +457,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>TC-UM-001</v>
+        <v>TC-UM-002</v>
       </c>
       <c r="B2" t="str">
-        <v>Verify successful manual user creation</v>
+        <v>Verify invite-based user onboarding</v>
       </c>
       <c r="C2" t="str">
         <v>User Management</v>
@@ -469,28 +469,28 @@
         <v>User Creation &amp; Invitations</v>
       </c>
       <c r="E2" t="str">
-        <v>FSD ID FS-RL-CF-04: Client admin can create users within license limits</v>
+        <v>FSD ID FS-RL-CF-04: Client admin can invite users to onboard.</v>
       </c>
       <c r="F2" t="str">
-        <v>To ensure that a Client admin can create a new user manually.</v>
+        <v>To ensure an invited user can complete the onboarding process via email.</v>
       </c>
       <c r="G2" t="str">
-        <v>1. Client admin is logged in.; 2. Permissions for user creation are granted.</v>
+        <v>1. Client admin is logged in.; 2. An invitation has been sent to the user's email.</v>
       </c>
       <c r="H2" t="str">
-        <v>['Full Name: Text (max 50 chars, alphabets and spaces only)', 'Email Address: Text (max 100 chars, must be unique and valid format)', 'Role: Dropdown (must exist in Role Management)']</v>
+        <v>['Email Address: Text (valid format and unique)', 'Link Expiry Time: DateTime (time-bound)']</v>
       </c>
       <c r="I2" t="str">
-        <v>1. Navigate to User Management; 2. Click on Add User and click New Internal User; 3. Enter first Name and last Name; 4. Enter Email Address; 5. Select Role; 6. Click on Save</v>
+        <v>1. Open the invite email; 2. Click the registration link; 3. Fill in required fields; 4. Set password; 5. Confirm password; 6. Click on Register</v>
       </c>
       <c r="J2" t="str">
-        <v>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Full Name field shows the entered value.; 4. Email Address field shows the entered value.; 5. Role dropdown reflects the chosen role.; 6. User is visible in the list with correct status with status Pending.; Overall: New user is listed in User Management with Pending status.</v>
+        <v>1. The email is opened and contains the registration link.; 2. User is redirected to the registration page.; 3. Fields are populated as per the email link.; 4. Password field reflects the entered value.; 5. Confirm Password field reflects the entered value.; 6. User status is updated to Active.; Overall: User successfully completes onboarding and logs in.</v>
       </c>
       <c r="K2" t="str">
-        <v>User appears in the user list with status Pending.</v>
+        <v>User is listed as Active in the user list.</v>
       </c>
       <c r="L2" t="str">
-        <v>User is not listed or has an incorrect status.</v>
+        <v>User fails to be activated or logs in unsuccessfully.</v>
       </c>
       <c r="M2" t="str">
         <v>Functional - Positive</v>
@@ -508,180 +508,12 @@
         <v>Yes</v>
       </c>
       <c r="R2" t="str">
-        <v>Final_x000d_</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>TC-UM-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Validate unique user email constraint</v>
-      </c>
-      <c r="C3" t="str">
-        <v>User Management</v>
-      </c>
-      <c r="D3" t="str">
-        <v>User Creation &amp; Invitations</v>
-      </c>
-      <c r="E3" t="str">
-        <v>FSD ID FS-RL-CF-04: Duplicate emails should not be allowed.</v>
-      </c>
-      <c r="F3" t="str">
-        <v>To ensure that the system prevents duplicate email entries.</v>
-      </c>
-      <c r="G3" t="str">
-        <v>1. A user with a registered email exists.; 2. Client admin is logged in.</v>
-      </c>
-      <c r="H3" t="str">
-        <v>['Email Address: Text (must not match any existing records)']</v>
-      </c>
-      <c r="I3" t="str">
-        <v>1. Navigate to User Management; 2. Click on Add User and click Add Internal User.; 3. Enter existing email address; 4. Click on Save</v>
-      </c>
-      <c r="J3" t="str">
-        <v>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Email field shows entered value.; 4. Error message displays: 'Email already exists.'; Overall: System prevents duplicate email from being registered.</v>
-      </c>
-      <c r="K3" t="str">
-        <v>User is not created, and relevant error is displayed.</v>
-      </c>
-      <c r="L3" t="str">
-        <v>User is created with duplicate email address.</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Functional - Negative</v>
-      </c>
-      <c r="N3" t="str">
-        <v>P1</v>
-      </c>
-      <c r="O3" t="str">
-        <v>Functional suitability</v>
-      </c>
-      <c r="P3" t="str">
-        <v>High</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Final_x000d_</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>TC-UM-003</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Verify role assignment to user</v>
-      </c>
-      <c r="C4" t="str">
-        <v>User Management</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Role Assignment</v>
-      </c>
-      <c r="E4" t="str">
-        <v>FSD ID FS-RL-CF-04: Roles must be assigned to users appropriately.</v>
-      </c>
-      <c r="F4" t="str">
-        <v>To ensure a Client admin can assign a role to a user.</v>
-      </c>
-      <c r="G4" t="str">
-        <v>1. User is created and exists in the system.; 2. Administrator is logged in and viewing user details.</v>
-      </c>
-      <c r="H4" t="str">
-        <v>['Role: Dropdown (must exist in Role Management)']</v>
-      </c>
-      <c r="I4" t="str">
-        <v>1. Navigate to User Management; 2.Click on the user and click on edit.; 3. Select role from Role dropdown; 4. Click on Save.</v>
-      </c>
-      <c r="J4" t="str">
-        <v>1. User Management page is displayed.; 2. User details are displayed.; 3. Role dropdown reflects the chosen role.; 4. User role is updated successfully.; Overall: User's assigned role reflects changes in the user list.</v>
-      </c>
-      <c r="K4" t="str">
-        <v>User role matches the assigned role.</v>
-      </c>
-      <c r="L4" t="str">
-        <v>User role is not updated in the user details.</v>
-      </c>
-      <c r="M4" t="str">
-        <v>Functional - Positive</v>
-      </c>
-      <c r="N4" t="str">
-        <v>P1</v>
-      </c>
-      <c r="O4" t="str">
-        <v>Functional suitability</v>
-      </c>
-      <c r="P4" t="str">
-        <v>Medium</v>
-      </c>
-      <c r="Q4" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Final_x000d_</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>TC-UM-004</v>
-      </c>
-      <c r="B5" t="str">
-        <v>Verify deactivation of a user</v>
-      </c>
-      <c r="C5" t="str">
-        <v>User Management</v>
-      </c>
-      <c r="D5" t="str">
-        <v>User Status Management</v>
-      </c>
-      <c r="E5" t="str">
-        <v>FSD ID FS-RL-CF-04: Deactivated users cannot access the platform.</v>
-      </c>
-      <c r="F5" t="str">
-        <v>To ensure a Client admin can deactivate a user.</v>
-      </c>
-      <c r="G5" t="str">
-        <v>1. User is active and exists in the system.; 2. Administrator is logged in.</v>
-      </c>
-      <c r="H5" t="str">
-        <v>['Status: Dropdown (must change from Active to Deactivated)']</v>
-      </c>
-      <c r="I5" t="str">
-        <v>1. Navigate to User Management; 2. Select the user; 3. Click on Deactivate</v>
-      </c>
-      <c r="J5" t="str">
-        <v>1. User Management page is displayed.; 2. User details are displayed.; 3. User status is updated to Deactivated.; Overall: User cannot sign in post-deactivation.</v>
-      </c>
-      <c r="K5" t="str">
-        <v>User status reflects Deactivated.</v>
-      </c>
-      <c r="L5" t="str">
-        <v>User status remains Active or the user can log in.</v>
-      </c>
-      <c r="M5" t="str">
-        <v>Functional - Positive</v>
-      </c>
-      <c r="N5" t="str">
-        <v>P1</v>
-      </c>
-      <c r="O5" t="str">
-        <v>Functional suitability</v>
-      </c>
-      <c r="P5" t="str">
-        <v>High</v>
-      </c>
-      <c r="Q5" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="R5" t="str">
         <v>Final</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: implement runtime payload injection, data redaction for sensitive fields, and enhance instruction normalization for verification and search flows
</commit_message>
<xml_diff>
--- a/input/test_flow.xlsx
+++ b/input/test_flow.xlsx
@@ -1,47 +1,409 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30126"/>
+  <workbookPr filterPrivacy="1"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_1CC9DCBF811AC26192DF0A613B3E9D1FDD803B56" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-60" yWindow="-60" windowWidth="15480" windowHeight="11640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
     <sheet name="in" sheetId="1" r:id="rId1"/>
   </sheets>
+  <calcPr calcId="171027"/>
+  <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
-<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
-<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
-  <metadataTypes count="1">
-    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
-  </metadataTypes>
-  <futureMetadata name="XLDAPR" count="1">
-    <bk>
-      <extLst>
-        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
-          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
-        </ext>
-      </extLst>
-    </bk>
-  </futureMetadata>
-  <cellMetadata count="1">
-    <bk>
-      <rc t="1" v="0"/>
-    </bk>
-  </cellMetadata>
-</metadata>
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="80">
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Case ID</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Case Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Module</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Sub-Module</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Basis</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Objective</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Preconditions</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Data Ref</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Steps</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Expected Results</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Pass Criteria</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Fail Criteria</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Test Type</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Priority</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>ISO 25010 Quality Characteristic</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Risk Level</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Automation Suitability</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+      </rPr>
+      <t>Scenario Source</t>
+    </r>
+  </si>
+  <si>
+    <t>TC-UM-001</t>
+  </si>
+  <si>
+    <t>Verify successful manual user creation</t>
+  </si>
+  <si>
+    <t>User Management</t>
+  </si>
+  <si>
+    <t>User Creation &amp; Invitations</t>
+  </si>
+  <si>
+    <t>FSD ID FS-RL-CF-04: Client admin can create users within license limits</t>
+  </si>
+  <si>
+    <t>To ensure that a Client admin can create a new user manually.</t>
+  </si>
+  <si>
+    <t>1. Client admin is logged in.; 2. Permissions for user creation are granted.</t>
+  </si>
+  <si>
+    <t>['Full Name: Text (max 50 chars, alphabets and spaces only)', 'Email Address: Text (max 100 chars, must be unique and valid format)', 'Role: Dropdown (must exist in Role Management)']</t>
+  </si>
+  <si>
+    <t>1. Navigate to User Management; 2. Click on Add User.; 3. click New Internal User.; 4. Enter first Name.; 5. Enter last Name.; 6. Enter Email Address.; 7. open the dropdown.; 8. Select Role.; 9. Click on Save.;</t>
+  </si>
+  <si>
+    <t>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Full Name field shows the entered value.; 4. Email Address field shows the entered value.; 5. Role dropdown reflects the chosen role.; 6. User is visible in the list with correct status with status Pending.; Overall: New user is listed in User Management with Pending status.</t>
+  </si>
+  <si>
+    <t>User appears in the user list with status Pending.</t>
+  </si>
+  <si>
+    <t>User is not listed or has an incorrect status.</t>
+  </si>
+  <si>
+    <t>Functional - Positive</t>
+  </si>
+  <si>
+    <t>P1</t>
+  </si>
+  <si>
+    <t>Functional suitability</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Yes</t>
+  </si>
+  <si>
+    <t>Final</t>
+  </si>
+  <si>
+    <t>TC-UM-002</t>
+  </si>
+  <si>
+    <t>Verify role assignment to user</t>
+  </si>
+  <si>
+    <t>Role Assignment</t>
+  </si>
+  <si>
+    <t>FSD ID FS-RL-CF-04: Roles must be assigned to users appropriately.</t>
+  </si>
+  <si>
+    <t>To ensure a Client admin can assign a role to a user.</t>
+  </si>
+  <si>
+    <t>1. User is created and exists in the system.; 2. Administrator is logged in and viewing user details.</t>
+  </si>
+  <si>
+    <t>['Role: Dropdown (must exist in Role Management)']</t>
+  </si>
+  <si>
+    <t>1. Navigate to User Management.; 2.Click on search.; 3. search the user by name or email.; 4. Click on the User.; 5. select edit.; 6. Open role dropdown.; 7. Select the role.; 6. Click on Save.</t>
+  </si>
+  <si>
+    <t>1. User Management page is displayed.; 2. User details are displayed.; 3. Role dropdown reflects the chosen role.; 4. User role is updated successfully.; Overall: User's assigned role reflects changes in the user list.</t>
+  </si>
+  <si>
+    <t>User role matches the assigned role.</t>
+  </si>
+  <si>
+    <t>User role is not updated in the user details.</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>TC-UM-003</t>
+  </si>
+  <si>
+    <t>Validate unique user email constraint</t>
+  </si>
+  <si>
+    <t>FSD ID FS-RL-CF-04: Duplicate emails should not be allowed.</t>
+  </si>
+  <si>
+    <t>To ensure that the system prevents duplicate email entries.</t>
+  </si>
+  <si>
+    <t>1. A user with a registered email exists.; 2. Client admin is logged in.</t>
+  </si>
+  <si>
+    <t>['Email Address: Text (must not match any existing records)']</t>
+  </si>
+  <si>
+    <t>1. Navigate to User Management; 2. Click on Add User; 3. click on new internal user.; 4. enter first name.; 5. enter last name.; 6. Enter existing email address; 7. Open role dropdown; 8.select the role; 9. Click on Save.</t>
+  </si>
+  <si>
+    <t>1. User Management page is displayed.; 2. Add User form is displayed.; 3. Email field shows entered value.; 4. Error message displays: 'Email already exists.'; Overall: System prevents duplicate email from being registered.</t>
+  </si>
+  <si>
+    <t>User is not created, and relevant error is displayed.</t>
+  </si>
+  <si>
+    <t>User is created with duplicate email address.</t>
+  </si>
+  <si>
+    <t>Functional - Negative</t>
+  </si>
+  <si>
+    <t>TC-UM-004</t>
+  </si>
+  <si>
+    <t>Verify deactivation of a user</t>
+  </si>
+  <si>
+    <t>User Status Management</t>
+  </si>
+  <si>
+    <t>FSD ID FS-RL-CF-04: Deactivated users cannot access the platform.</t>
+  </si>
+  <si>
+    <t>To ensure a Client admin can deactivate a user.</t>
+  </si>
+  <si>
+    <t>1. User is active and exists in the system.; 2. Administrator is logged in.</t>
+  </si>
+  <si>
+    <t>['Status: Dropdown (must change from Active to Deactivated)']</t>
+  </si>
+  <si>
+    <t>1. Navigate to User Management; 2. Click on search.; 3. search the user by name or email id.; 4. Click on the user.; 5. Click on Deactivate.; 6. enter the comment in add comments.; 7. click on deactivate.</t>
+  </si>
+  <si>
+    <t>1. User Management page is displayed.; 2. User details are displayed.; 3. User status is updated to Deactivated.; Overall: User cannot sign in post-deactivation.</t>
+  </si>
+  <si>
+    <t>User status reflects Deactivated.</t>
+  </si>
+  <si>
+    <t>User status remains Active or the user can log in.</t>
+  </si>
+  <si>
+    <t>TC-UM-005</t>
+  </si>
+  <si>
+    <t>Verify reactivation of a user</t>
+  </si>
+  <si>
+    <t>FSD ID FS-RL-CF-04: Reactivated users can access the platform.</t>
+  </si>
+  <si>
+    <t>To ensure a Client admin can reactivate a user.</t>
+  </si>
+  <si>
+    <t>1. User is deactivated and exists in the system.; 2. Administrator is logged in.</t>
+  </si>
+  <si>
+    <t>['Status: Dropdown (must change from Deactivated to Active)']</t>
+  </si>
+  <si>
+    <t>1. Navigate to User Management; 2. Click on search.; 3. search the user by name or email id.; 4. Click on the user.; 5. Click on Reactivate.; 6. enter the comment in add comments.; 7. click on reactivate.</t>
+  </si>
+  <si>
+    <t>1. User Management page is displayed.; 2. User details are displayed.; 3. User status is updated to Active.; Overall: User can sign in post-reactivation.</t>
+  </si>
+  <si>
+    <t>User status reflects Active.</t>
+  </si>
+  <si>
+    <t>User status remains Deactivated.</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
-  <numFmts count="1">
-    <numFmt numFmtId="56" formatCode="&quot;上午/下午 &quot;hh&quot;時&quot;mm&quot;分&quot;ss&quot;秒 &quot;"/>
-  </numFmts>
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2">
     <font>
-      <sz val="12"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -65,13 +427,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -396,124 +766,353 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:R2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:R6"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="33.28515625" customWidth="1"/>
+    <col min="3" max="3" width="17.7109375" customWidth="1"/>
+    <col min="4" max="4" width="24.5703125" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>Test Case ID</v>
-      </c>
-      <c r="B1" t="str">
-        <v>Test Case Name</v>
-      </c>
-      <c r="C1" t="str">
-        <v>Module</v>
-      </c>
-      <c r="D1" t="str">
-        <v>Sub-Module</v>
-      </c>
-      <c r="E1" t="str">
-        <v>Test Basis</v>
-      </c>
-      <c r="F1" t="str">
-        <v>Test Objective</v>
-      </c>
-      <c r="G1" t="str">
-        <v>Preconditions</v>
-      </c>
-      <c r="H1" t="str">
-        <v>Test Data Ref</v>
-      </c>
-      <c r="I1" t="str">
-        <v>Test Steps</v>
-      </c>
-      <c r="J1" t="str">
-        <v>Expected Results</v>
-      </c>
-      <c r="K1" t="str">
-        <v>Pass Criteria</v>
-      </c>
-      <c r="L1" t="str">
-        <v>Fail Criteria</v>
-      </c>
-      <c r="M1" t="str">
-        <v>Test Type</v>
-      </c>
-      <c r="N1" t="str">
-        <v>Priority</v>
-      </c>
-      <c r="O1" t="str">
-        <v>ISO 25010 Quality Characteristic</v>
-      </c>
-      <c r="P1" t="str">
-        <v>Risk Level</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>Automation Suitability</v>
-      </c>
-      <c r="R1" t="str">
-        <v>Scenario Source</v>
+    <row r="1" spans="1:18">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+      <c r="K1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
+      <c r="N1" t="s">
+        <v>13</v>
+      </c>
+      <c r="O1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" t="s">
+        <v>17</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>TC-UM-002</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Verify invite-based user onboarding</v>
-      </c>
-      <c r="C2" t="str">
-        <v>User Management</v>
-      </c>
-      <c r="D2" t="str">
-        <v>User Creation &amp; Invitations</v>
-      </c>
-      <c r="E2" t="str">
-        <v>FSD ID FS-RL-CF-04: Client admin can invite users to onboard.</v>
-      </c>
-      <c r="F2" t="str">
-        <v>To ensure an invited user can complete the onboarding process via email.</v>
-      </c>
-      <c r="G2" t="str">
-        <v>1. Client admin is logged in.; 2. An invitation has been sent to the user's email.</v>
-      </c>
-      <c r="H2" t="str">
-        <v>['Email Address: Text (valid format and unique)', 'Link Expiry Time: DateTime (time-bound)']</v>
-      </c>
-      <c r="I2" t="str">
-        <v>1. Open the invite email; 2. Click the registration link; 3. Fill in required fields; 4. Set password; 5. Confirm password; 6. Click on Register</v>
-      </c>
-      <c r="J2" t="str">
-        <v>1. The email is opened and contains the registration link.; 2. User is redirected to the registration page.; 3. Fields are populated as per the email link.; 4. Password field reflects the entered value.; 5. Confirm Password field reflects the entered value.; 6. User status is updated to Active.; Overall: User successfully completes onboarding and logs in.</v>
-      </c>
-      <c r="K2" t="str">
-        <v>User is listed as Active in the user list.</v>
-      </c>
-      <c r="L2" t="str">
-        <v>User fails to be activated or logs in unsuccessfully.</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Functional - Positive</v>
-      </c>
-      <c r="N2" t="str">
-        <v>P1</v>
-      </c>
-      <c r="O2" t="str">
-        <v>Functional suitability</v>
-      </c>
-      <c r="P2" t="str">
-        <v>High</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="R2" t="str">
-        <v>Final</v>
+    <row r="2" spans="1:18">
+      <c r="A2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F2" t="s">
+        <v>23</v>
+      </c>
+      <c r="G2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" t="s">
+        <v>26</v>
+      </c>
+      <c r="J2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K2" t="s">
+        <v>28</v>
+      </c>
+      <c r="L2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M2" t="s">
+        <v>30</v>
+      </c>
+      <c r="N2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O2" t="s">
+        <v>32</v>
+      </c>
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>34</v>
+      </c>
+      <c r="R2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18">
+      <c r="A3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" t="s">
+        <v>40</v>
+      </c>
+      <c r="G3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H3" t="s">
+        <v>42</v>
+      </c>
+      <c r="I3" t="s">
+        <v>43</v>
+      </c>
+      <c r="J3" t="s">
+        <v>44</v>
+      </c>
+      <c r="K3" t="s">
+        <v>45</v>
+      </c>
+      <c r="L3" t="s">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>30</v>
+      </c>
+      <c r="N3" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P3" t="s">
+        <v>47</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>34</v>
+      </c>
+      <c r="R3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18">
+      <c r="A4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B4" t="s">
+        <v>49</v>
+      </c>
+      <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" t="s">
+        <v>52</v>
+      </c>
+      <c r="H4" t="s">
+        <v>53</v>
+      </c>
+      <c r="I4" t="s">
+        <v>54</v>
+      </c>
+      <c r="J4" t="s">
+        <v>55</v>
+      </c>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
+      <c r="L4" t="s">
+        <v>57</v>
+      </c>
+      <c r="M4" t="s">
+        <v>58</v>
+      </c>
+      <c r="N4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O4" t="s">
+        <v>32</v>
+      </c>
+      <c r="P4" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>34</v>
+      </c>
+      <c r="R4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18">
+      <c r="A5" t="s">
+        <v>59</v>
+      </c>
+      <c r="B5" t="s">
+        <v>60</v>
+      </c>
+      <c r="C5" t="s">
+        <v>20</v>
+      </c>
+      <c r="D5" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" t="s">
+        <v>62</v>
+      </c>
+      <c r="F5" t="s">
+        <v>63</v>
+      </c>
+      <c r="G5" t="s">
+        <v>64</v>
+      </c>
+      <c r="H5" t="s">
+        <v>65</v>
+      </c>
+      <c r="I5" t="s">
+        <v>66</v>
+      </c>
+      <c r="J5" t="s">
+        <v>67</v>
+      </c>
+      <c r="K5" t="s">
+        <v>68</v>
+      </c>
+      <c r="L5" t="s">
+        <v>69</v>
+      </c>
+      <c r="M5" t="s">
+        <v>30</v>
+      </c>
+      <c r="N5" t="s">
+        <v>31</v>
+      </c>
+      <c r="O5" t="s">
+        <v>32</v>
+      </c>
+      <c r="P5" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>34</v>
+      </c>
+      <c r="R5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18">
+      <c r="A6" t="s">
+        <v>70</v>
+      </c>
+      <c r="B6" t="s">
+        <v>71</v>
+      </c>
+      <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6" t="s">
+        <v>61</v>
+      </c>
+      <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G6" t="s">
+        <v>74</v>
+      </c>
+      <c r="H6" t="s">
+        <v>75</v>
+      </c>
+      <c r="I6" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" t="s">
+        <v>77</v>
+      </c>
+      <c r="K6" t="s">
+        <v>78</v>
+      </c>
+      <c r="L6" t="s">
+        <v>79</v>
+      </c>
+      <c r="M6" t="s">
+        <v>30</v>
+      </c>
+      <c r="N6" t="s">
+        <v>31</v>
+      </c>
+      <c r="O6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P6" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q6" t="s">
+        <v>34</v>
+      </c>
+      <c r="R6" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:R2"/>
-  </ignoredErrors>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>